<commit_message>
Lançar feriados, adiantamento e vale-transporte do GENECIR em setembro
Feriados de 07/09 e 08/09 trabalhados (2 salários-dia, R$ 108,06) na
aba de ponto, adiantamento de R$ 500,00 em 09/09 e R$ 270,00 de
vale-transporte. A folha de setembro passa a aceitar vales e compra de
vale-transporte pela configuração da loja.

Fica registrado que, se 08/09 for feriado municipal, o fator de DSR das
três lojas muda de 5/25 para 6/24.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_ARRAIAL_pgto_05-10-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_ARRAIAL_pgto_05-10-2026.xlsx
@@ -2607,7 +2607,7 @@
       </c>
       <c r="K24" s="30" t="inlineStr">
         <is>
-          <t>PREENCHER com os vales adiantados durante setembro.</t>
+          <t xml:space="preserve">PREENCHER com os vales adiantados durante setembro. </t>
         </is>
       </c>
     </row>
@@ -2933,7 +2933,7 @@
       </c>
       <c r="K35" s="30" t="inlineStr">
         <is>
-          <t>PREENCHER com as passagens compradas para outubro/2026.</t>
+          <t xml:space="preserve">PREENCHER com as passagens compradas. </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Considerar o feriado municipal de 08/09 no DSR de setembro
Com o feriado municipal de 08/09, setembro passa a ter 6 dias de
repouso (4 domingos mais 07/09 e 08/09) sobre 24 dias úteis: fator de
DSR 0,25 em vez de 0,20, nas três lojas. Passagem de trabalho e README
atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_ARRAIAL_pgto_05-10-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_SETEMBRO_2026_ARRAIAL_pgto_05-10-2026.xlsx
@@ -800,7 +800,7 @@
       <c r="A20" s="4" t="inlineStr"/>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>DSR de setembro/2026: 4 domingos + o feriado de 07/09 ÷ 25 dias úteis = fator 0,200000</t>
+          <t>DSR de setembro/2026: 4 domingos + os feriados de 07/09 e 08/09 (municipal) = 6 ÷ 24 dias úteis = fator 0,250000</t>
         </is>
       </c>
     </row>
@@ -1135,11 +1135,11 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Domingos: 06, 13, 20 e 27/09/2026, mais o feriado de 07/09 (segunda-feira). CONFERIR feriados municipais.</t>
+          <t>Domingos: 06, 13, 20 e 27/09/2026, mais os feriados de 07/09 (Independência, segunda) e 08/09 (municipal, terça).</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="K12" s="30" t="inlineStr">
         <is>
-          <t>Cálculo: (comissão total + horas extras) × (4 domingos + feriado 07/09) ÷ 25 dias úteis de setembro/2026.</t>
+          <t>Cálculo: (comissão total + horas extras) × (4 domingos + feriados de 07/09 e 08/09) ÷ 24 dias úteis de setembro/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>